<commit_message>
Handle incomplete correlation matrices from Excel
</commit_message>
<xml_diff>
--- a/przykladowy_excel.xlsx
+++ b/przykladowy_excel.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\source\repos\Metoda-Hellwiga\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="M:\repos_new\Metoda-Hellwiga\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{766BDED4-20DD-48A6-B991-BFA58E6A06E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{772C555B-5B6C-4F6E-A906-1FAD04778C75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4770" yWindow="360" windowWidth="23340" windowHeight="10755" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1380" yWindow="2220" windowWidth="12690" windowHeight="11010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="6">
   <si>
     <t>y</t>
   </si>
@@ -87,7 +87,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normalny" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -387,146 +387,164 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="1">
-        <v>1</v>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
       </c>
       <c r="B2" s="1">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1">
         <v>0.57760299999999998</v>
       </c>
-      <c r="C2" s="1">
+      <c r="D2" s="1">
         <v>0.86505799999999999</v>
       </c>
-      <c r="D2" s="1">
+      <c r="E2" s="1">
         <v>0.48166999999999999</v>
       </c>
-      <c r="E2" s="1">
+      <c r="F2" s="1">
         <v>0.86777599999999999</v>
       </c>
-      <c r="F2" s="1">
+      <c r="G2" s="1">
         <v>0.82841200000000004</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="1">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="1">
         <v>0.57760299999999998</v>
       </c>
-      <c r="B3" s="1">
-        <v>1</v>
-      </c>
       <c r="C3" s="1">
+        <v>1</v>
+      </c>
+      <c r="D3" s="1">
         <v>0.79284299999999996</v>
       </c>
-      <c r="D3" s="1">
+      <c r="E3" s="1">
         <v>0.264075</v>
       </c>
-      <c r="E3" s="1">
+      <c r="F3" s="1">
         <v>0.64499799999999996</v>
       </c>
-      <c r="F3" s="1">
+      <c r="G3" s="1">
         <v>0.101383</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="1">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="1">
         <v>0.86505799999999999</v>
       </c>
-      <c r="B4" s="1">
+      <c r="C4" s="1">
         <v>0.79284299999999996</v>
       </c>
-      <c r="C4" s="1">
-        <v>1</v>
-      </c>
       <c r="D4" s="1">
+        <v>1</v>
+      </c>
+      <c r="E4" s="1">
         <v>0.32916400000000001</v>
       </c>
-      <c r="E4" s="1">
+      <c r="F4" s="1">
         <v>0.86178299999999997</v>
       </c>
-      <c r="F4" s="1">
+      <c r="G4" s="1">
         <v>0.58533000000000002</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="1">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="1">
         <v>0.48166999999999999</v>
       </c>
-      <c r="B5" s="1">
+      <c r="C5" s="1">
         <v>0.264075</v>
       </c>
-      <c r="C5" s="1">
+      <c r="D5" s="1">
         <v>0.32916400000000001</v>
       </c>
-      <c r="D5" s="1">
-        <v>1</v>
-      </c>
       <c r="E5" s="1">
+        <v>1</v>
+      </c>
+      <c r="F5" s="1">
         <v>0.17324300000000001</v>
       </c>
-      <c r="F5" s="1">
+      <c r="G5" s="1">
         <v>0.51317199999999996</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="1">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="1">
         <v>0.86777599999999999</v>
       </c>
-      <c r="B6" s="1">
+      <c r="C6" s="1">
         <v>0.64499799999999996</v>
       </c>
-      <c r="C6" s="1">
+      <c r="D6" s="1">
         <v>0.86178299999999997</v>
       </c>
-      <c r="D6" s="1">
+      <c r="E6" s="1">
         <v>0.17324300000000001</v>
       </c>
-      <c r="E6" s="1">
-        <v>1</v>
-      </c>
       <c r="F6" s="1">
+        <v>1</v>
+      </c>
+      <c r="G6" s="1">
         <v>0.61691099999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="1">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="1">
         <v>0.82841200000000004</v>
       </c>
-      <c r="B7" s="1">
+      <c r="C7" s="1">
         <v>0.101383</v>
       </c>
-      <c r="C7" s="1">
+      <c r="D7" s="1">
         <v>0.58533000000000002</v>
       </c>
-      <c r="D7" s="1">
+      <c r="E7" s="1">
         <v>0.51317199999999996</v>
       </c>
-      <c r="E7" s="1">
+      <c r="F7" s="1">
         <v>0.61691099999999999</v>
       </c>
-      <c r="F7" s="1">
+      <c r="G7" s="1">
         <v>1</v>
       </c>
     </row>

</xml_diff>